<commit_message>
Localize spreadsheet columns and outputs to Spanish
</commit_message>
<xml_diff>
--- a/data/raw/cierre_agricola/aguacate_2024.xlsx
+++ b/data/raw/cierre_agricola/aguacate_2024.xlsx
@@ -431,47 +431,47 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Unnamed: 0_level_0 Unnamed: 0_level_1</t>
+          <t>numero</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Entidad Entidad</t>
+          <t>entidad</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Superficie (ha) Sembrada</t>
+          <t>superficie_sembrada_ha</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Superficie (ha) Cosechada</t>
+          <t>superficie_cosechada_ha</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Superficie (ha) Siniestrada</t>
+          <t>superficie_siniestrada_ha</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Producción Producción</t>
+          <t>produccion</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Rendimiento (udm/ha) Rendimiento (udm/ha)</t>
+          <t>rendimiento_udm_ha</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>PMR ($/udm) PMR ($/udm)</t>
+          <t>pmr_mxn_udm</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Valor Producción (miles de Pesos) Valor Producción (miles de Pesos)</t>
+          <t>valor_produccion_miles_pesos</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Localize spreadsheet columns and outputs to Spanish (#8)
</commit_message>
<xml_diff>
--- a/data/raw/cierre_agricola/aguacate_2024.xlsx
+++ b/data/raw/cierre_agricola/aguacate_2024.xlsx
@@ -431,47 +431,47 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Unnamed: 0_level_0 Unnamed: 0_level_1</t>
+          <t>numero</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Entidad Entidad</t>
+          <t>entidad</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Superficie (ha) Sembrada</t>
+          <t>superficie_sembrada_ha</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Superficie (ha) Cosechada</t>
+          <t>superficie_cosechada_ha</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Superficie (ha) Siniestrada</t>
+          <t>superficie_siniestrada_ha</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Producción Producción</t>
+          <t>produccion</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Rendimiento (udm/ha) Rendimiento (udm/ha)</t>
+          <t>rendimiento_udm_ha</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>PMR ($/udm) PMR ($/udm)</t>
+          <t>pmr_mxn_udm</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Valor Producción (miles de Pesos) Valor Producción (miles de Pesos)</t>
+          <t>valor_produccion_miles_pesos</t>
         </is>
       </c>
     </row>

</xml_diff>